<commit_message>
FixBug: Summary without Grouping NullReferenceException
</commit_message>
<xml_diff>
--- a/tests/Templates/GroupTagTests_Simple_Empty.xlsx
+++ b/tests/Templates/GroupTagTests_Simple_Empty.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Address</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>&lt;&lt;sum default="0"&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;sum default="2"&gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1189,7 @@
       </c>
       <c r="I13" s="24"/>
       <c r="J13" s="25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>